<commit_message>
Cập nhật hoàn thiện bài tập Day 03
</commit_message>
<xml_diff>
--- a/data/expense_tracker.xlsx
+++ b/data/expense_tracker.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,21 +622,93 @@
           <t>Ăn uống</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Bữa tối</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="b">
         <v>0</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>2026-09-13T15:32:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ăn uống</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bữa tối</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-13T17:39:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ăn uống</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Bữa tối</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-13T17:39:07</t>
         </is>
       </c>
     </row>

</xml_diff>